<commit_message>
Add work setup section and tool logos; US spelling; layout fixes
- My Work Setup section with workspace photo (screen contents blurred)
- Official logos in the Tools & Platforms section
- American English spelling and month-first dates across site and workbook
- Administrative Support and Basic Accounting Admin in Where I Help Most
- Wider avatar crop; cleaner layout for the design samples card

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/Ali-Puchero-EA-Operations-Toolkit.xlsx
+++ b/files/Ali-Puchero-EA-Operations-Toolkit.xlsx
@@ -66,7 +66,7 @@
     <t>Calculated</t>
   </si>
   <si>
-    <t>Grey cells contain formulas and update automatically. Please don’t type over them.</t>
+    <t>Gray cells contain formulas and update automatically. Please don’t type over them.</t>
   </si>
   <si>
     <t>Header</t>
@@ -219,7 +219,7 @@
     <t>Roles and responsibilities for 12 recurring activities, with a built-in check that every row has exactly one accountable owner.</t>
   </si>
   <si>
-    <t>All clients, people, invoices, leads and figures in this workbook are fictitious placeholders created to demonstrate these systems. Any resemblance to real organisations is coincidental.</t>
+    <t>All clients, people, invoices, leads and figures in this workbook are fictitious placeholders created to demonstrate these systems. Any resemblance to real organizations is coincidental.</t>
   </si>
   <si>
     <t>Operations Dashboard</t>
@@ -357,25 +357,25 @@
     <t>Includes 4 invoices that are not yet due.</t>
   </si>
   <si>
-    <t>Two accounts escalated to Finance on 27 Oct.</t>
-  </si>
-  <si>
-    <t>Westfield v2 proposal due 31 Oct.</t>
+    <t>Two accounts escalated to Finance on Oct 27.</t>
+  </si>
+  <si>
+    <t>Westfield v2 proposal due Oct 31.</t>
   </si>
   <si>
     <t>Owners reminded on Thursday.</t>
   </si>
   <si>
-    <t>Session 3 certificates going out by 3 Nov.</t>
-  </si>
-  <si>
-    <t>Westfield onboarding started 30 Oct.</t>
+    <t>Session 3 certificates going out by Nov 3.</t>
+  </si>
+  <si>
+    <t>Westfield onboarding started Oct 30.</t>
   </si>
   <si>
     <t>Highlights</t>
   </si>
   <si>
-    <t>•  Q4 board pack outline approved; financial summary due 2 Nov.</t>
+    <t>•  Q4 board pack outline approved; financial summary due Nov 2.</t>
   </si>
   <si>
     <t>•  Sydney trip booked; client dinner, one meeting and the airport taxi still to confirm.</t>
@@ -393,13 +393,13 @@
     <t>•  Approve revised Westfield scope before it goes to the client.</t>
   </si>
   <si>
-    <t>•  Confirm attendees for the 14 Nov planning day.</t>
+    <t>•  Confirm attendees for the Nov 14 planning day.</t>
   </si>
   <si>
     <t>Priorities next week</t>
   </si>
   <si>
-    <t>•  Finalise and send the board pack.</t>
+    <t>•  Finalize and send the board pack.</t>
   </si>
   <si>
     <t>•  Issue Session 3 CPD certificates.</t>
@@ -905,7 +905,7 @@
     <t>Send the welcome email and onboarding pack</t>
   </si>
   <si>
-    <t>Personalise the template; attach engagement letter and client information form.</t>
+    <t>Personalize the template; attach engagement letter and client information form.</t>
   </si>
   <si>
     <t>Email</t>
@@ -1103,7 +1103,7 @@
     <t>Over 45 days: escalate to the manager</t>
   </si>
   <si>
-    <t>Summarise the history (dates, contacts, promises) in one email.</t>
+    <t>Summarize the history (dates, contacts, promises) in one email.</t>
   </si>
   <si>
     <t>Escalation sent</t>
@@ -1130,7 +1130,7 @@
     <t>Tone stays courteous at every stage; no threats or fees unless approved by Finance.</t>
   </si>
   <si>
-    <t>Promised payment dates are diarised and checked the following day.</t>
+    <t>Promised payment dates are added to the calendar and checked the following day.</t>
   </si>
   <si>
     <t>Client disputes the amount or the work: stop reminders and pass to Finance the same day.</t>
@@ -1335,7 +1335,7 @@
     <t>In progress</t>
   </si>
   <si>
-    <t>Finance summary due from Finance Lead on 2 Nov</t>
+    <t>Finance summary due from Finance Lead on Nov 2</t>
   </si>
   <si>
     <t>T-002</t>
@@ -1356,7 +1356,7 @@
     <t>T-003</t>
   </si>
   <si>
-    <t>Send onboarding pack to Harbourline Accounting</t>
+    <t>Send onboarding pack to Harborline Accounting</t>
   </si>
   <si>
     <t>Client onboarding</t>
@@ -1377,7 +1377,7 @@
     <t>Waiting on others</t>
   </si>
   <si>
-    <t>Reminder sent 27 Oct</t>
+    <t>Reminder sent Oct 27</t>
   </si>
   <si>
     <t>T-005</t>
@@ -1563,10 +1563,10 @@
     <t>INV-1041</t>
   </si>
   <si>
-    <t>Harbourline Accounting</t>
-  </si>
-  <si>
-    <t>accounts@harbourlineacc.example.com</t>
+    <t>Harborline Accounting</t>
+  </si>
+  <si>
+    <t>accounts@harborlineacco.example.com</t>
   </si>
   <si>
     <t>INV-1042</t>
@@ -1767,7 +1767,7 @@
     <t>Practice Manager</t>
   </si>
   <si>
-    <t>Website enquiry</t>
+    <t>Website inquiry</t>
   </si>
   <si>
     <t>Monthly bookkeeping</t>
@@ -1878,7 +1878,7 @@
     <t>Sunbeam Early Learning</t>
   </si>
   <si>
-    <t>Centre Director</t>
+    <t>Center Director</t>
   </si>
   <si>
     <t>Bookkeeping</t>
@@ -2040,7 +2040,7 @@
     <t>Account Mgr, Client CFO, EA</t>
   </si>
   <si>
-    <t>Quarterly review set for 5 Nov</t>
+    <t>Quarterly review set for Nov 5</t>
   </si>
   <si>
     <t>Send quarterly review invite + agenda</t>
@@ -2073,7 +2073,7 @@
     <t>Update SOP-04 with new routine</t>
   </si>
   <si>
-    <t>Planning day on 14 Nov</t>
+    <t>Planning day on Nov 14</t>
   </si>
   <si>
     <t>Confirm venue and catering numbers</t>
@@ -2205,7 +2205,7 @@
     <t>J. Santos</t>
   </si>
   <si>
-    <t>jsantos@harbourlineacc.example.com</t>
+    <t>jsantos@harborlineacco.example.com</t>
   </si>
   <si>
     <t>Y</t>
@@ -2412,7 +2412,7 @@
     <t>Sample itinerary for a three-day client trip, with confirmations, costs and a budget check.</t>
   </si>
   <si>
-    <t>Traveller</t>
+    <t>Traveler</t>
   </si>
   <si>
     <t>Client visits + industry conference</t>
@@ -2427,7 +2427,7 @@
     <t>Dates</t>
   </si>
   <si>
-    <t>4–6 November 2026</t>
+    <t>November 4–6, 2026</t>
   </si>
   <si>
     <t>Time</t>
@@ -2496,7 +2496,7 @@
     <t>Check-in, 2 nights, quiet room requested, breakfast included</t>
   </si>
   <si>
-    <t>Harbour Hotel</t>
+    <t>Harbor Hotel</t>
   </si>
   <si>
     <t>HH-554019</t>
@@ -2616,7 +2616,7 @@
     <t>Sources</t>
   </si>
   <si>
-    <t>Vendor documentation and help centres; free trials; independent user reviews (e.g. G2, Capterra); team feedback sessions.</t>
+    <t>Vendor documentation and help centers; free trials; independent user reviews (e.g. G2, Capterra); team feedback sessions.</t>
   </si>
   <si>
     <t>Top-scoring option</t>
@@ -2637,7 +2637,7 @@
     <t>Approve the trial → set up workspace and templates (EA) → team walkthrough (30 min) → review after 14 days.</t>
   </si>
   <si>
-    <t>Delivered on 23 Oct 2026; trial approved at the 26 Oct leadership meeting (see Meeting Actions).</t>
+    <t>Delivered on Oct 23, 2026; trial approved at the Oct 26 leadership meeting (see Meeting Actions).</t>
   </si>
   <si>
     <t>Research: Project Management Tool Evaluation</t>
@@ -2790,7 +2790,7 @@
     <t>CRM → client follow-up</t>
   </si>
   <si>
-    <t>New enquiry received</t>
+    <t>New inquiry received</t>
   </si>
   <si>
     <t>Create the lead with source and service interest</t>
@@ -2805,7 +2805,7 @@
     <t>Lead created</t>
   </si>
   <si>
-    <t>Assign stage and owner; add notes from the enquiry</t>
+    <t>Assign stage and owner; add notes from the inquiry</t>
   </si>
   <si>
     <t>Stage set</t>
@@ -3048,7 +3048,7 @@
     <t>Booking status</t>
   </si>
   <si>
-    <t>Cancelled</t>
+    <t>Canceled</t>
   </si>
   <si>
     <t>Edit these lists to change the drop-down options used across the workbook. Stage probabilities (column F) drive the weighted pipeline in CRM Pipeline.</t>
@@ -3059,7 +3059,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="dd mmm yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0;-0;&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
@@ -10886,8 +10886,8 @@
     </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="str">
-        <f>"Live summary of every tracker · as of "&amp;DAY(AsOfDate)&amp;"/"&amp;MONTH(AsOfDate)&amp;"/"&amp;YEAR(AsOfDate)</f>
-        <v>Live summary of every tracker · as of 30/10/2026</v>
+        <f>"Live summary of every tracker · as of "&amp;MONTH(AsOfDate)&amp;"/"&amp;DAY(AsOfDate)&amp;"/"&amp;YEAR(AsOfDate)</f>
+        <v>Live summary of every tracker · as of 10/30/2026</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -11883,8 +11883,8 @@
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="str">
-        <f>"Week ending "&amp;DAY(AsOfDate)&amp;"/"&amp;MONTH(AsOfDate)&amp;"/"&amp;YEAR(AsOfDate)&amp;" · prepared by Ali Puchero, Executive Assistant"</f>
-        <v>Week ending 30/10/2026 · prepared by Ali Puchero, Executive Assistant</v>
+        <f>"Week ending "&amp;MONTH(AsOfDate)&amp;"/"&amp;DAY(AsOfDate)&amp;"/"&amp;YEAR(AsOfDate)&amp;" · prepared by Ali Puchero, Executive Assistant"</f>
+        <v>Week ending 10/30/2026 · prepared by Ali Puchero, Executive Assistant</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>

</xml_diff>